<commit_message>
Update to include multi-page figure layout generateion (landscape only)
</commit_message>
<xml_diff>
--- a/Figures_Individual_Int_By_Scenario.xlsx
+++ b/Figures_Individual_Int_By_Scenario.xlsx
@@ -16884,7 +16884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AA184"/>
+  <dimension ref="B2:Y184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.6" customWidth="1" min="1" max="1"/>
@@ -17100,11 +17100,6 @@
       <c r="W2" s="2" t="n"/>
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="3" t="n"/>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>Existing 20XX Traffc Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="B3" s="4" t="n"/>
@@ -17836,11 +17831,6 @@
       <c r="W33" s="2" t="n"/>
       <c r="X33" s="2" t="n"/>
       <c r="Y33" s="3" t="n"/>
-      <c r="AA33" t="inlineStr">
-        <is>
-          <t>Existing 20XX Traffc Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="B34" s="4" t="n"/>
@@ -18572,11 +18562,6 @@
       <c r="W64" s="2" t="n"/>
       <c r="X64" s="2" t="n"/>
       <c r="Y64" s="3" t="n"/>
-      <c r="AA64" t="inlineStr">
-        <is>
-          <t>Existing 20XX Traffc Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="B65" s="4" t="n"/>
@@ -19310,11 +19295,6 @@
       <c r="W95" s="2" t="n"/>
       <c r="X95" s="2" t="n"/>
       <c r="Y95" s="3" t="n"/>
-      <c r="AA95" t="inlineStr">
-        <is>
-          <t>Existing 20XX Traffc Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="B96" s="4" t="n"/>
@@ -20032,11 +20012,6 @@
       <c r="W126" s="2" t="n"/>
       <c r="X126" s="2" t="n"/>
       <c r="Y126" s="3" t="n"/>
-      <c r="AA126" t="inlineStr">
-        <is>
-          <t>Existing 20XX Traffc Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="127">
       <c r="B127" s="4" t="n"/>
@@ -20770,11 +20745,6 @@
       <c r="W157" s="2" t="n"/>
       <c r="X157" s="2" t="n"/>
       <c r="Y157" s="3" t="n"/>
-      <c r="AA157" t="inlineStr">
-        <is>
-          <t>Existing 20XX Traffc Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="158">
       <c r="B158" s="4" t="n"/>
@@ -21611,7 +21581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AA184"/>
+  <dimension ref="B2:Y184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.6" customWidth="1" min="1" max="1"/>
@@ -21827,11 +21797,6 @@
       <c r="W2" s="2" t="n"/>
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="3" t="n"/>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>No-Build 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="B3" s="4" t="n"/>
@@ -22565,11 +22530,6 @@
       <c r="W33" s="2" t="n"/>
       <c r="X33" s="2" t="n"/>
       <c r="Y33" s="3" t="n"/>
-      <c r="AA33" t="inlineStr">
-        <is>
-          <t>No-Build 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="B34" s="4" t="n"/>
@@ -23301,11 +23261,6 @@
       <c r="W64" s="2" t="n"/>
       <c r="X64" s="2" t="n"/>
       <c r="Y64" s="3" t="n"/>
-      <c r="AA64" t="inlineStr">
-        <is>
-          <t>No-Build 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="B65" s="4" t="n"/>
@@ -24039,11 +23994,6 @@
       <c r="W95" s="2" t="n"/>
       <c r="X95" s="2" t="n"/>
       <c r="Y95" s="3" t="n"/>
-      <c r="AA95" t="inlineStr">
-        <is>
-          <t>No-Build 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="B96" s="4" t="n"/>
@@ -24761,11 +24711,6 @@
       <c r="W126" s="2" t="n"/>
       <c r="X126" s="2" t="n"/>
       <c r="Y126" s="3" t="n"/>
-      <c r="AA126" t="inlineStr">
-        <is>
-          <t>No-Build 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="127">
       <c r="B127" s="4" t="n"/>
@@ -25499,11 +25444,6 @@
       <c r="W157" s="2" t="n"/>
       <c r="X157" s="2" t="n"/>
       <c r="Y157" s="3" t="n"/>
-      <c r="AA157" t="inlineStr">
-        <is>
-          <t>No-Build 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="158">
       <c r="B158" s="4" t="n"/>
@@ -26340,7 +26280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AA184"/>
+  <dimension ref="B2:Y184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.6" customWidth="1" min="1" max="1"/>
@@ -26556,11 +26496,6 @@
       <c r="W2" s="2" t="n"/>
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="3" t="n"/>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>Build 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="B3" s="4" t="n"/>
@@ -27294,11 +27229,6 @@
       <c r="W33" s="2" t="n"/>
       <c r="X33" s="2" t="n"/>
       <c r="Y33" s="3" t="n"/>
-      <c r="AA33" t="inlineStr">
-        <is>
-          <t>Build 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="B34" s="4" t="n"/>
@@ -28030,11 +27960,6 @@
       <c r="W64" s="2" t="n"/>
       <c r="X64" s="2" t="n"/>
       <c r="Y64" s="3" t="n"/>
-      <c r="AA64" t="inlineStr">
-        <is>
-          <t>Build 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="B65" s="4" t="n"/>
@@ -28768,11 +28693,6 @@
       <c r="W95" s="2" t="n"/>
       <c r="X95" s="2" t="n"/>
       <c r="Y95" s="3" t="n"/>
-      <c r="AA95" t="inlineStr">
-        <is>
-          <t>Build 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="B96" s="4" t="n"/>
@@ -29490,11 +29410,6 @@
       <c r="W126" s="2" t="n"/>
       <c r="X126" s="2" t="n"/>
       <c r="Y126" s="3" t="n"/>
-      <c r="AA126" t="inlineStr">
-        <is>
-          <t>Build 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="127">
       <c r="B127" s="4" t="n"/>
@@ -30228,11 +30143,6 @@
       <c r="W157" s="2" t="n"/>
       <c r="X157" s="2" t="n"/>
       <c r="Y157" s="3" t="n"/>
-      <c r="AA157" t="inlineStr">
-        <is>
-          <t>Build 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="158">
       <c r="B158" s="4" t="n"/>
@@ -31069,7 +30979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AA184"/>
+  <dimension ref="B2:Y184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.6" customWidth="1" min="1" max="1"/>
@@ -31285,11 +31195,6 @@
       <c r="W2" s="2" t="n"/>
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="3" t="n"/>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>Remove 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="B3" s="4" t="n"/>
@@ -32023,11 +31928,6 @@
       <c r="W33" s="2" t="n"/>
       <c r="X33" s="2" t="n"/>
       <c r="Y33" s="3" t="n"/>
-      <c r="AA33" t="inlineStr">
-        <is>
-          <t>Remove 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="B34" s="4" t="n"/>
@@ -32759,11 +32659,6 @@
       <c r="W64" s="2" t="n"/>
       <c r="X64" s="2" t="n"/>
       <c r="Y64" s="3" t="n"/>
-      <c r="AA64" t="inlineStr">
-        <is>
-          <t>Remove 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="B65" s="4" t="n"/>
@@ -33497,11 +33392,6 @@
       <c r="W95" s="2" t="n"/>
       <c r="X95" s="2" t="n"/>
       <c r="Y95" s="3" t="n"/>
-      <c r="AA95" t="inlineStr">
-        <is>
-          <t>Remove 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="B96" s="4" t="n"/>
@@ -34219,11 +34109,6 @@
       <c r="W126" s="2" t="n"/>
       <c r="X126" s="2" t="n"/>
       <c r="Y126" s="3" t="n"/>
-      <c r="AA126" t="inlineStr">
-        <is>
-          <t>Remove 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="127">
       <c r="B127" s="4" t="n"/>
@@ -34957,11 +34842,6 @@
       <c r="W157" s="2" t="n"/>
       <c r="X157" s="2" t="n"/>
       <c r="Y157" s="3" t="n"/>
-      <c r="AA157" t="inlineStr">
-        <is>
-          <t>Remove 20XX Traffic Volumes</t>
-        </is>
-      </c>
     </row>
     <row r="158">
       <c r="B158" s="4" t="n"/>

</xml_diff>